<commit_message>
last set of updates prior experiments
</commit_message>
<xml_diff>
--- a/cognite/neat/rules/examples/skos-rules.xlsx
+++ b/cognite/neat/rules/examples/skos-rules.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/niva/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Secondary/repos/neat/cognite/neat/rules/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2629C31B-F964-6D46-AD13-C5DC3EE8E3FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91C0E979-C8B8-5947-A55A-E5F7FF93ED3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34400" yWindow="500" windowWidth="34400" windowHeight="28300" xr2:uid="{DC5DAD83-861A-3547-A43E-AF26CFD744F6}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="70">
   <si>
     <t>Class</t>
   </si>
@@ -297,10 +297,6 @@
     <t>Concept</t>
   </si>
   <si>
-    <t>A SKOS concept scheme can be viewed as an aggregation of one or more SKOS concepts. Semantic relationships (links) between those concepts may also be viewed as part of a concept scheme. This definition is, however, meant to be suggestive rather than restrictive, and there is some flexibility in the formal data model stated below.
-The notion of a concept scheme is useful when dealing with data from an unknown source, and when dealing with data that describes two or more different knowledge organization systems.</t>
-  </si>
-  <si>
     <t>Collection</t>
   </si>
   <si>
@@ -319,10 +315,6 @@
     <t>http://www.w3.org/2004/02/skos/core#OrderedCollection</t>
   </si>
   <si>
-    <t>SKOS concept collections are labeled and/or ordered groups of SKOS concepts.
-Collections are useful where a group of concepts shares something in common, and it is convenient to group them under a common label, or where some concepts can be placed in a meaningful order.</t>
-  </si>
-  <si>
     <t>prefLabel</t>
   </si>
   <si>
@@ -359,12 +351,6 @@
     <t>hasTopConcept</t>
   </si>
   <si>
-    <t>A SKOS concept can be viewed as an idea or notion; a unit of thought. However, what constitutes a unit of thought is subjective, and this definition is meant to be suggestive, rather than restrictive.
-The notion of a SKOS concept is useful when describing the conceptual or intellectual structure of a knowledge organization system, and when referring to specific ideas or meanings established within a KOS.
-Note that, because SKOS is designed to be a vehicle for representing semi-formal KOS, such as thesauri and classification schemes, a certain amount of flexibility has been built in to the formal definition of this class.
-A SKOS concept can be viewed as an idea or notion; a unit of thought. However, what constitutes a unit of thought is subjective, and this definition is meant to be suggestive, rather than restrictive.</t>
-  </si>
-  <si>
     <t>license</t>
   </si>
   <si>
@@ -405,9 +391,6 @@
   </si>
   <si>
     <t>external_id</t>
-  </si>
-  <si>
-    <t>wind_energy_taxonomy</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1010,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>29</v>
@@ -1035,10 +1018,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -1083,10 +1066,10 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1131,42 +1114,36 @@
       <c r="A3" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="22" t="s">
-        <v>58</v>
-      </c>
+      <c r="B3" s="22"/>
       <c r="C3" s="28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="22" t="s">
-        <v>38</v>
-      </c>
+      <c r="B4" s="22"/>
       <c r="C4" s="27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>45</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B5" s="22"/>
       <c r="C5" s="27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1231,10 +1208,10 @@
         <v>34</v>
       </c>
       <c r="H2" s="32" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I2" s="32" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -1242,7 +1219,7 @@
         <v>37</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13" t="s">
@@ -1259,7 +1236,7 @@
         <v>http://www.w3.org/2004/02/skos/core#prefLabel</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I3" t="str">
         <f>"skos:" &amp; A3 &amp; "(skos:" &amp; B3 &amp; ")"</f>
@@ -1271,7 +1248,7 @@
         <v>37</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13" t="s">
@@ -1288,7 +1265,7 @@
         <v>http://www.w3.org/2004/02/skos/core#definition</v>
       </c>
       <c r="H4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I4" t="str">
         <f t="shared" ref="I4:I15" si="1">"skos:" &amp; A4 &amp; "(skos:" &amp; B4 &amp; ")"</f>
@@ -1300,7 +1277,7 @@
         <v>37</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13" t="s">
@@ -1315,7 +1292,7 @@
         <v>http://www.w3.org/2004/02/skos/core#altLabel</v>
       </c>
       <c r="H5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I5" t="str">
         <f t="shared" si="1"/>
@@ -1327,7 +1304,7 @@
         <v>37</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13" t="s">
@@ -1344,7 +1321,7 @@
         <v>http://www.w3.org/2004/02/skos/core#inScheme</v>
       </c>
       <c r="H6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="1"/>
@@ -1356,7 +1333,7 @@
         <v>37</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="13" t="s">
@@ -1373,7 +1350,7 @@
         <v>http://www.w3.org/2004/02/skos/core#topConceptOf</v>
       </c>
       <c r="H7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I7" t="str">
         <f t="shared" si="1"/>
@@ -1385,7 +1362,7 @@
         <v>37</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13" t="s">
@@ -1400,7 +1377,7 @@
         <v>http://www.w3.org/2004/02/skos/core#broader</v>
       </c>
       <c r="H8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I8" t="str">
         <f t="shared" si="1"/>
@@ -1412,7 +1389,7 @@
         <v>37</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="13" t="s">
@@ -1427,7 +1404,7 @@
         <v>http://www.w3.org/2004/02/skos/core#narrower</v>
       </c>
       <c r="H9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I9" t="str">
         <f t="shared" si="1"/>
@@ -1439,11 +1416,11 @@
         <v>37</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E10" s="13">
         <v>0</v>
@@ -1454,7 +1431,7 @@
         <v>http://www.w3.org/2004/02/skos/core#related</v>
       </c>
       <c r="H10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I10" t="str">
         <f t="shared" si="1"/>
@@ -1466,11 +1443,11 @@
         <v>37</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E11" s="13">
         <v>0</v>
@@ -1481,7 +1458,7 @@
         <v>http://www.w3.org/2004/02/skos/core#closeMatch</v>
       </c>
       <c r="H11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I11" t="str">
         <f t="shared" si="1"/>
@@ -1493,11 +1470,11 @@
         <v>37</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E12" s="13">
         <v>0</v>
@@ -1508,7 +1485,7 @@
         <v>http://www.w3.org/2004/02/skos/core#exactMatch</v>
       </c>
       <c r="H12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I12" t="str">
         <f t="shared" si="1"/>
@@ -1520,11 +1497,11 @@
         <v>37</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E13" s="13">
         <v>0</v>
@@ -1535,7 +1512,7 @@
         <v>http://www.w3.org/2004/02/skos/core#relatedMatch</v>
       </c>
       <c r="H13" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I13" t="str">
         <f t="shared" si="1"/>
@@ -1547,7 +1524,7 @@
         <v>36</v>
       </c>
       <c r="B14" s="29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C14" s="29"/>
       <c r="D14" s="29" t="s">
@@ -1562,7 +1539,7 @@
         <v>http://www.w3.org/2004/02/skos/core#hasTopConcept</v>
       </c>
       <c r="H14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I14" t="str">
         <f t="shared" si="1"/>
@@ -1574,7 +1551,7 @@
         <v>36</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" s="29"/>
       <c r="D15" s="29" t="s">
@@ -1591,7 +1568,7 @@
         <v>http://www.w3.org/2004/02/skos/core#prefLabel</v>
       </c>
       <c r="H15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I15" t="str">
         <f t="shared" si="1"/>
@@ -1620,7 +1597,7 @@
         <v>http://purl.org/dc/terms/description</v>
       </c>
       <c r="H16" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I16" t="str">
         <f>"skos:" &amp; A16 &amp; "(dct:" &amp; B16 &amp; ")"</f>
@@ -1632,7 +1609,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C17" s="29"/>
       <c r="D17" s="29" t="s">
@@ -1649,7 +1626,7 @@
         <v>http://purl.org/dc/terms/title</v>
       </c>
       <c r="H17" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I17" t="str">
         <f>"skos:" &amp; A17 &amp; "(dct:" &amp; B17 &amp; ")"</f>
@@ -1661,11 +1638,11 @@
         <v>36</v>
       </c>
       <c r="B18" s="29" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C18" s="29"/>
       <c r="D18" s="29" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E18" s="29">
         <v>1</v>
@@ -1678,7 +1655,7 @@
         <v>http://purl.org/dc/terms/created</v>
       </c>
       <c r="H18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I18" t="str">
         <f t="shared" ref="I18:I24" si="4">"skos:" &amp; A18 &amp; "(dct:" &amp; B18 &amp; ")"</f>
@@ -1690,11 +1667,11 @@
         <v>36</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C19" s="29"/>
       <c r="D19" s="29" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E19" s="29">
         <v>1</v>
@@ -1707,7 +1684,7 @@
         <v>http://purl.org/dc/terms/modified</v>
       </c>
       <c r="H19" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I19" t="str">
         <f t="shared" si="4"/>
@@ -1719,7 +1696,7 @@
         <v>36</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C20" s="29"/>
       <c r="D20" s="29" t="s">
@@ -1736,7 +1713,7 @@
         <v>http://purl.org/dc/terms/hasVersion</v>
       </c>
       <c r="H20" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I20" t="str">
         <f t="shared" si="4"/>
@@ -1763,7 +1740,7 @@
         <v>http://purl.org/dc/terms/creator</v>
       </c>
       <c r="H21" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I21" t="str">
         <f t="shared" si="4"/>
@@ -1790,7 +1767,7 @@
         <v>http://purl.org/dc/terms/contributor</v>
       </c>
       <c r="H22" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I22" t="str">
         <f t="shared" si="4"/>
@@ -1802,7 +1779,7 @@
         <v>36</v>
       </c>
       <c r="B23" s="29" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C23" s="29"/>
       <c r="D23" s="29" t="s">
@@ -1819,7 +1796,7 @@
         <v>http://purl.org/dc/terms/license</v>
       </c>
       <c r="H23" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I23" t="str">
         <f t="shared" si="4"/>
@@ -1831,7 +1808,7 @@
         <v>36</v>
       </c>
       <c r="B24" s="29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C24" s="29"/>
       <c r="D24" s="29" t="s">
@@ -1848,7 +1825,7 @@
         <v>http://purl.org/dc/terms/rights</v>
       </c>
       <c r="H24" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I24" t="str">
         <f t="shared" si="4"/>
@@ -1940,17 +1917,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="52b81742-33c2-40cc-b790-7e45219c7334">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f0bd56e2-4aae-4be1-b2c1-2cc2e5553e4d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100579BE8B05CE7034EB45A78AA68378F2E" ma:contentTypeVersion="13" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="3e5fff67086aedf62c65cb7b025de975">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="52b81742-33c2-40cc-b790-7e45219c7334" xmlns:ns3="f0bd56e2-4aae-4be1-b2c1-2cc2e5553e4d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9250e7a2aff0c3bef49f240901aeee7" ns2:_="" ns3:_="">
     <xsd:import namespace="52b81742-33c2-40cc-b790-7e45219c7334"/>
@@ -2173,6 +2139,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="52b81742-33c2-40cc-b790-7e45219c7334">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f0bd56e2-4aae-4be1-b2c1-2cc2e5553e4d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A58FD28A-F2DD-4C04-BF54-9689FD79BAB6}">
   <ds:schemaRefs>
@@ -2182,23 +2159,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{036D60ED-F4C4-492F-BC12-2AE5A093DE00}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="f0bd56e2-4aae-4be1-b2c1-2cc2e5553e4d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="52b81742-33c2-40cc-b790-7e45219c7334"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{502A94D1-4307-442E-AABE-D52193DC6B44}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2215,4 +2175,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{036D60ED-F4C4-492F-BC12-2AE5A093DE00}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="f0bd56e2-4aae-4be1-b2c1-2cc2e5553e4d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="52b81742-33c2-40cc-b790-7e45219c7334"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>